<commit_message>
Ingest customer ODS: Powermax 65, LinuxCNC+Mesa, X1600xY2500, critical-speed finding
- README: customer spec table from Plasma Table Constraints.ods; correct torch
  (Powermax 65, customer supplies) and control stack (LinuxCNC Qtplasmac + SheetCAM +
  Mesa 7i76e + THCAD-5/10); envelope 1000x2000 min / X1600xY2500 outer (the chat's
  1700x1700 was material on hand, not the envelope).
- spreadsheet/constraints.xlsx: Inputs now carries ODS customer spec + feature list;
  B4 longest axis -> 2500 mm (governing span); critical-speed formula corrected to the
  standard Nc=K*D/L^2*1e7 with K (15.1 fixed-supported) and D (25 mm) as cross-checkable
  inputs. Verdict: ballscrew critical speed FAILS at 2500 mm span for 15 m/min plasma;
  rack has no critical-speed limit -> rack preferred for the long axis.
</commit_message>
<xml_diff>
--- a/spreadsheet/constraints.xlsx
+++ b/spreadsheet/constraints.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +69,13 @@
     <font>
       <color rgb="00333333"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +117,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5B8F"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -139,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,6 +178,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -713,22 +726,21 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Ballscrew critical speed (1700 bed)</t>
+          <t>Ballscrew critical speed (2500 mm span)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>750 rpm (20mm lead)</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>1394 rpm (20mm dia, 2000mm)</t>
-        </is>
+          <t>750 rpm (20 mm lead @ 15 m/min)</t>
+        </is>
+      </c>
+      <c r="C9" s="4">
+        <f>ROUND(Inputs!$B$53*Inputs!$B$54*10000000/(Inputs!$B$4+Inputs!$B$22)^2,0) rpm</f>
+        <v/>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>1.9x</t>
+          <t>FAIL vs 50% rule</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -876,7 +888,7 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Every constraint passes with &gt;=1.5x margin. The 2000 N is a Z-only load and is comfortably handled by a self-locking 2.5mm lead screw + 51217 thrust bearing + 2x HGH20. The X/Y decision is therefore NOT capability — it is precision/backlash (ballscrew) vs simplicity/cost/full-1700mm-length (rack &amp; pinion). Two real constraints the bed size introduces: (1) the 900 rpm encoder cap forces a ballscrew lead &gt;= ~17 mm to reach 15 m/min; (2) a 20 mm lead on a ~2000 mm span needs &gt;=25 mm dia (or a mid-span bearing) to stay under 50% of critical speed. A rack has neither limit.</t>
+          <t>BOTTOM LINE — corrected for the customer's REAL longest axis (2500 mm, from the ODS): at that span a ballscrew's critical speed is the BINDING constraint for 15 m/min plasma — every ballscrew lead needs &gt;750 rpm, which exceeds even 100% of critical speed (K=15.1, D=25, L=2800 -&gt; ~480 rpm). The RACK has no critical-speed limit, so for the LONG axis the rack is the safer 15 m/min choice; a ballscrew works only if you go larger-diameter, add a mid-span bearing, or accept slower rapids. Force and torque still pass easily everywhere (2000 N is Z-only). Edit K and D (yellow) to test your actual screw.</t>
         </is>
       </c>
     </row>
@@ -899,7 +911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -928,11 +940,11 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Bed size X (working)</t>
+          <t>Longest travel axis (screw span basis)</t>
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>1700</v>
+        <v>2500</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -948,11 +960,13 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Bed size Y (working)</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>1700</v>
+          <t>Min sheet to cut (customer)</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>1000 x 2000</t>
+        </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -973,7 +987,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Hypertherm 45 (45 A)</t>
+          <t>Hypertherm POWERMAX 65 (customer supplies, w/ CPC)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1035,7 +1049,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>plasma 15 m/min; light engrave/emboss/brass-gear (slow)</t>
+          <t>plasma+THC 15 m/min; light engrave/emboss/mill/drill (slow)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1406,6 +1420,266 @@
       <c r="D29" s="10" t="inlineStr">
         <is>
           <t>3 mm steel typical</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>CUSTOMER REQUIREMENTS  (Plasma Table Constraints.ods, 2026-10-21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Outer maximum dimensions (X, Y)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1600 x 2500</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>customer 'outer max'</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Min sheet to cut</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1000 x 2000</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>'able to cut at least 1000x2000 sheets'</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Available (customer)</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>customer '1700mm'</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Torch (customer buys)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Powermax 65 + CPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Control software</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LinuxCNC Qtplasmac + SheetCAM (local at machine)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Motion controller</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Mesa 7i76e (Ethernet FPGA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>THC — touch-off</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Mesa THCAD-5 (ohmic sensing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>THC — real-time</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Mesa THCAD-10 (voltage sensing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>EMI/EMI concern</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>high — plasma cutter generates lots of electrical noise</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
+        <is>
+          <t>DESIRED FEATURES (customer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Plasma cutting with THC + water table</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Break-away feature (part collision protection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Scribing tool (pneumatic or electric)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Drilling small holes + spot drilling</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>High / adjustable Z-axis (for cutting curved surfaces)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Cut at least 1000x2000 sheets (bigger is better)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Light milling (ballscrew vs belts — customer's own suggestion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>4th axis for tube plasma cutting</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>More features e.g. gear tooth cutter</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="20" t="inlineStr">
+        <is>
+          <t>BALLSCREW CRITICAL SPEED  (Nc = K * D / L^2 * 1e7 rpm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>End-support factor K</t>
+        </is>
+      </c>
+      <c r="B53" s="22" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>fixed-free 3.4 | sup-sup 9.7 | fixed-supp 15.1 | fixed-fixed 21.9 (K=(beta*L)^2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Ballscrew diameter D (nominal)</t>
+        </is>
+      </c>
+      <c r="B54" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>larger lead -&gt; larger dia; scale to your screw</t>
         </is>
       </c>
     </row>
@@ -1788,7 +2062,7 @@
         <v/>
       </c>
       <c r="J5" s="17">
-        <f>ROUND(307000000*20/I5^2,0)</f>
+        <f>ROUND(Inputs!$B$53*Inputs!$B$54*10000000/I5^2,0)</f>
         <v/>
       </c>
       <c r="K5" s="17">
@@ -1843,7 +2117,7 @@
         <v/>
       </c>
       <c r="J6" s="17">
-        <f>ROUND(307000000*20/I6^2,0)</f>
+        <f>ROUND(Inputs!$B$53*Inputs!$B$54*10000000/I6^2,0)</f>
         <v/>
       </c>
       <c r="K6" s="17">
@@ -1898,7 +2172,7 @@
         <v/>
       </c>
       <c r="J7" s="17">
-        <f>ROUND(307000000*20/I7^2,0)</f>
+        <f>ROUND(Inputs!$B$53*Inputs!$B$54*10000000/I7^2,0)</f>
         <v/>
       </c>
       <c r="K7" s="17">
@@ -1953,7 +2227,7 @@
         <v/>
       </c>
       <c r="J8" s="17">
-        <f>ROUND(307000000*20/I8^2,0)</f>
+        <f>ROUND(Inputs!$B$53*Inputs!$B$54*10000000/I8^2,0)</f>
         <v/>
       </c>
       <c r="K8" s="17">
@@ -2008,7 +2282,7 @@
         <v/>
       </c>
       <c r="J9" s="17">
-        <f>ROUND(307000000*20/I9^2,0)</f>
+        <f>ROUND(Inputs!$B$53*Inputs!$B$54*10000000/I9^2,0)</f>
         <v/>
       </c>
       <c r="K9" s="17">

</xml_diff>

<commit_message>
Add water table + table height lift (2026-10-21 design request)
- spreadsheet/constraints.xlsx: new Water-Table sheet (live formulas) + 11 new
  Inputs (footprint, water depth, structure mass, pulley MA, CW safety factor,
  pump flow, pins, cable, pin shear). Verdicts: CW<empty (no self-lift when
  drained), manual force <=1000 N, cable SF>=10, pin SF>=5 — all PASS with
  defaults (~78 kg manual lift full of water, cable SF 18x, pin SF 9.5x,
  fill ~6 min, gravity drain).
- README: water table + height lift section (telescoping sq-tube guides,
  pulley/cable/counterweight assist, pin-fixed set heights, passive safety
  stop), verdict table, decisions-log entry.
</commit_message>
<xml_diff>
--- a/spreadsheet/constraints.xlsx
+++ b/spreadsheet/constraints.xlsx
@@ -12,6 +12,7 @@
     <sheet name="XY-Force" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Drive-XY" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Z-Drill" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Water-Table" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +75,27 @@
       <color rgb="00666666"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="FF666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+    </font>
+    <font>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -122,6 +142,11 @@
         <fgColor rgb="002F5B8F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -149,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +206,12 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -570,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -896,6 +927,112 @@
     <row r="18"/>
     <row r="19"/>
     <row r="20"/>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>WATER TABLE + TABLE HEIGHT LIFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Water load (1700x1700x100 mm)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>≈ 290 kg / 2845 N</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>+ ~250 kg structure = ~540 kg full (see Water-Table sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Counterweight max (passive safety)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>≤ 0.9 x EMPTY weight</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>guarantees a drained table can't self-lift into the plasma head</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Manual effort (full, 4:1 MA)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>≈ 80 kg equiv</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>(full − CW)/4 — one person workable</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cable / pins safety factor</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>≥ 10 / ≥ 5</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>6 mm steel cable, 2x M12 pins at set positions</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Fill / drain</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>≈ 6 min / gravity</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>50 L/min basic pump; sump drain</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>SAFETY NOTE — empty-water crash mode:</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>If the counterweight exceeded the EMPTY table weight, a drained table would self-lift and slam into the plasma head. Passive fix: CW &lt; 0.9 x empty weight. Pins then hold every set position with the cable slacked — no power or brake needed at rest.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
@@ -911,13 +1048,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1680,6 +1817,230 @@
       <c r="D54" s="21" t="inlineStr">
         <is>
           <t>larger lead -&gt; larger dia; scale to your screw</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
+          <t>WATER TABLE + TABLE HEIGHT LIFT  (2026-10-21 design request)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Water table footprint L</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D57" s="26" t="inlineStr">
+        <is>
+          <t>customer bed 1700x1700; set to work envelope if different</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Water table footprint W</t>
+        </is>
+      </c>
+      <c r="B58" s="25" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Water depth above workpiece</t>
+        </is>
+      </c>
+      <c r="B59" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D59" s="26" t="inlineStr">
+        <is>
+          <t>typical water-table jet depth; adjust if needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Table structure mass (frame+top+gantry)</t>
+        </is>
+      </c>
+      <c r="B60" s="25" t="n">
+        <v>250</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D60" s="26" t="inlineStr">
+        <is>
+          <t>ESTIMATE — weigh the built frame and update</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Lift mechanical advantage (pulley purchase)</t>
+        </is>
+      </c>
+      <c r="B61" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="26" t="inlineStr">
+        <is>
+          <t>4:1 = 4 rope parts; 2:1 also viable</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Counterweight safety factor (of empty weight)</t>
+        </is>
+      </c>
+      <c r="B62" s="25" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="26" t="inlineStr">
+        <is>
+          <t>CW &lt; empty weight so a DRAINED table can never self-lift into the torch</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Fill pump flow</t>
+        </is>
+      </c>
+      <c r="B63" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>L/min</t>
+        </is>
+      </c>
+      <c r="D63" s="26" t="inlineStr">
+        <is>
+          <t>basic pump (customer spec)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Fixing pins (set positions)</t>
+        </is>
+      </c>
+      <c r="B64" s="25" t="inlineStr">
+        <is>
+          <t>M12 x 2</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D64" s="26" t="inlineStr">
+        <is>
+          <t>pins take static load; cable can slack off</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Steel cable dia</t>
+        </is>
+      </c>
+      <c r="B65" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D65" s="26" t="inlineStr">
+        <is>
+          <t>verify with vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Cable min breaking load</t>
+        </is>
+      </c>
+      <c r="B66" s="25" t="n">
+        <v>24000</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D66" s="26" t="inlineStr">
+        <is>
+          <t>6 mm steel cable typical; verify with vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Pin shear capacity each</t>
+        </is>
+      </c>
+      <c r="B67" s="25" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D67" s="26" t="inlineStr">
+        <is>
+          <t>M12 steel shear ~25-40 kN; verify material</t>
         </is>
       </c>
     </row>
@@ -2860,4 +3221,467 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>WATER TABLE + TABLE HEIGHT LIFT  (live calcs — inputs on the Inputs sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>Water cools the kerf/workpiece (prevents warping), damps the plasma arc. Table raise/lower for access, counterweight-assisted, pin-fixed at set heights. X/Y fixed to table; plasma head keeps its own large Z travel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>--- WATER LOAD ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Water volume</t>
+        </is>
+      </c>
+      <c r="B5" s="28">
+        <f>Inputs!B57*Inputs!B58*Inputs!B59/1000000000</f>
+        <v/>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>m^3</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>L x W x depth</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Water mass</t>
+        </is>
+      </c>
+      <c r="B6" s="28">
+        <f>B5*1000</f>
+        <v/>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>1000 kg/m^3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Water weight</t>
+        </is>
+      </c>
+      <c r="B7" s="28">
+        <f>B6*9.81</f>
+        <v/>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Empty table weight</t>
+        </is>
+      </c>
+      <c r="B8" s="28">
+        <f>Inputs!B60*9.81</f>
+        <v/>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>structure mass x g</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FULL table weight (lifting load)</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
+        <f>B7+B8</f>
+        <v/>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>what the lift system sees</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>--- COUNTERWEIGHT + ASSIST ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Max counterweight (passive safety)</t>
+        </is>
+      </c>
+      <c r="B11" s="28">
+        <f>Inputs!B62*Inputs!B60*9.81</f>
+        <v/>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>0.9 x EMPTY weight -&gt; drained table can NEVER self-lift into the torch</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Counterweight mass</t>
+        </is>
+      </c>
+      <c r="B12" s="28">
+        <f>B11/9.81</f>
+        <v/>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>hang on the opposite rope</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Residual manual force (table FULL)</t>
+        </is>
+      </c>
+      <c r="B13" s="28">
+        <f>(B9-B11)/Inputs!B61</f>
+        <v/>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>(full - CW) / MA — what the operator feels</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = lifting equivalent</t>
+        </is>
+      </c>
+      <c r="B14" s="28">
+        <f>B13/9.81</f>
+        <v/>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>should feel ~&lt;100 kg for one person</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Manual force (table EMPTY, lowering)</t>
+        </is>
+      </c>
+      <c r="B15" s="28">
+        <f>B11/Inputs!B61</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>CW alone drives lowering of empty bed — keep small, controlled</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>--- SAFETY VERDICTS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>PASS: CW &lt; empty weight (no self-lift when drained)</t>
+        </is>
+      </c>
+      <c r="B17" s="28">
+        <f>IF(B11&lt;B8,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>the 'bed crashing into workpiece if empty of water' protection — passive, no power/brake</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PASS: manual force (full) &lt;= 1000 N</t>
+        </is>
+      </c>
+      <c r="B18" s="28">
+        <f>IF(B13&lt;=1000,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>raise stays one-person workable; else increase MA or CW</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Cable working load per rope part</t>
+        </is>
+      </c>
+      <c r="B19" s="28">
+        <f>B9/Inputs!B61</f>
+        <v/>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>full weight shared over MA rope parts (CW unloads the rest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PASS: cable safety factor &gt;= 10</t>
+        </is>
+      </c>
+      <c r="B20" s="28">
+        <f>IF(Inputs!B66/B19&gt;=10,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>breaking / working</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>PASS: pin safety factor &gt;= 5</t>
+        </is>
+      </c>
+      <c r="B21" s="28">
+        <f>IF(Inputs!B67*2/B9&gt;=5,"PASS","FAIL")</f>
+        <v/>
+      </c>
+      <c r="D21" s="26" t="inlineStr">
+        <is>
+          <t>2 x pin shear vs full weight — pins hold every set position</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>--- FILL / DRAIN ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Fill time</t>
+        </is>
+      </c>
+      <c r="B23" s="28">
+        <f>B5*1000/Inputs!B63</f>
+        <v/>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>volume / pump flow (basic pump)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Drain</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>gravity + sump</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
+        <is>
+          <t>drain hose to floor drain; optional drain pump for moving</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>--- MECHANICAL DESIGN (notes from user 2026-10-21) ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Guides</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>telescoping square tube: smaller tube inside main column, bearings guide it</t>
+        </is>
+      </c>
+      <c r="D26" s="26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Lift</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>pulley + steel cable + counterweight (assist, not full lift)</t>
+        </is>
+      </c>
+      <c r="D27" s="26" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Positioning</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>pins fix the table at set heights; cable can slack off — no power/brake at rest</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CW limit + mechanical detents: drained bed can only rest at pinned heights, can't self-lift</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Axes</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>X/Y fixed to table — whole table raises; plasma head keeps its own LARGE Z travel</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Spreadsheet Water-Table: append OPERATING POLICY (drain-before-raise, job shop, manual tool change)
</commit_message>
<xml_diff>
--- a/spreadsheet/constraints.xlsx
+++ b/spreadsheet/constraints.xlsx
@@ -3229,7 +3229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3681,6 +3681,37 @@
       </c>
       <c r="D30" s="26" t="inlineStr"/>
     </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>OPERATING POLICY (2026-10-21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Drain BEFORE raising</t>
+        </is>
+      </c>
+      <c r="B32" s="26" t="inlineStr">
+        <is>
+          <t>full table only LOWERS (CW-assisted); drained table is light and easy to raise</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>One-off job shop</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
+        <is>
+          <t>not a production machine — manual fixturing per process; manual tool change for now, ATC possible later</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>